<commit_message>
add grid tests and tests on Doublewell
</commit_message>
<xml_diff>
--- a/mcjax/process/metric_results.xlsx
+++ b/mcjax/process/metric_results.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,20 +457,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>delta_logZ</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>sinkhorn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>wasserstein</t>
         </is>
@@ -479,273 +484,715 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>doublewell</t>
+          <t>1d</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
+          <t>Kullback-Leibler</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
           <t>dds</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>0.4418703715006511</v>
-      </c>
       <c r="D2" t="n">
-        <v>0.3867161571979523</v>
+        <v>0.02234990398089091</v>
       </c>
       <c r="E2" t="n">
-        <v>1.065415342648824</v>
+        <v>0.008191856555640697</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.08570227178739848</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>mcd</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>4.051440238952637</v>
-      </c>
       <c r="D3" t="n">
-        <v>0.3335832456747691</v>
+        <v>0.002582561292607958</v>
       </c>
       <c r="E3" t="n">
-        <v>1.16065506140391</v>
+        <v>0.006039514672011137</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.04851661423498668</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>pis</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>1.320449352264404</v>
-      </c>
       <c r="D4" t="n">
-        <v>0.370587944984436</v>
+        <v>0.2139455825090408</v>
       </c>
       <c r="E4" t="n">
-        <v>1.128479823470116</v>
+        <v>0.007560619929184516</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1327734203520207</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>doublewell2</t>
-        </is>
-      </c>
+      <c r="A5" s="1" t="n"/>
       <c r="B5" s="1" t="inlineStr">
         <is>
+          <t>Log-variance</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
           <t>dds</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>3.84380849202474</v>
-      </c>
       <c r="D5" t="n">
-        <v>7.31148624420166</v>
+        <v>0.02123528532683849</v>
       </c>
       <c r="E5" t="n">
-        <v>7.292523225148519</v>
+        <v>0.006751975665489833</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.08162500043235728</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>mcd</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>5.863048553466797</v>
-      </c>
       <c r="D6" t="n">
-        <v>7.319493770599365</v>
+        <v>0.001702137863806759</v>
       </c>
       <c r="E6" t="n">
-        <v>7.3003249168396</v>
+        <v>0.005845834811528523</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.04191472911149455</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n"/>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>pis</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>3.950328826904297</v>
-      </c>
       <c r="D7" t="n">
-        <v>7.50787369410197</v>
+        <v>34.39225323994955</v>
       </c>
       <c r="E7" t="n">
-        <v>7.490129470825195</v>
+        <v>2.434566259384155</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.45810746017271</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>funnel</t>
+          <t>doublewell</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
+          <t>Kullback-Leibler</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
           <t>dds</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>0.252522071202596</v>
-      </c>
       <c r="D8" t="n">
-        <v>0.8421547015508016</v>
+        <v>2.733012994130453</v>
       </c>
       <c r="E8" t="n">
-        <v>6.877715428670247</v>
+        <v>4.250979661941528</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.788908629742651</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>mcd</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>0.1519577503204346</v>
-      </c>
       <c r="D9" t="n">
-        <v>0.7756073474884033</v>
+        <v>5.895169734954834</v>
       </c>
       <c r="E9" t="n">
-        <v>6.711217403411865</v>
+        <v>0.3406601846218109</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.644682632533477</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>pis</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>1.360313713550568</v>
-      </c>
       <c r="D10" t="n">
-        <v>0.9259290993213654</v>
+        <v>0.1741339365641276</v>
       </c>
       <c r="E10" t="n">
-        <v>7.078276872634888</v>
+        <v>0.4348956942558289</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.8734950738541555</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>gmmfixed</t>
-        </is>
-      </c>
+      <c r="A11" s="1" t="n"/>
       <c r="B11" s="1" t="inlineStr">
         <is>
+          <t>Log-variance</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
           <t>dds</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>0.5782348016897837</v>
-      </c>
       <c r="D11" t="n">
-        <v>0.07451121260722478</v>
+        <v>1.664091110229492</v>
       </c>
       <c r="E11" t="n">
-        <v>1.275897304217021</v>
+        <v>0.357625941435496</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.092607790618223</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>mcd</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>0.5899389982223511</v>
-      </c>
       <c r="D12" t="n">
-        <v>0.08400427053372066</v>
+        <v>7.808188438415527</v>
       </c>
       <c r="E12" t="n">
-        <v>1.903177579243978</v>
+        <v>0.3409054577350616</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.8966926320625664</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>pis</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>3.083451827367147</v>
-      </c>
       <c r="D13" t="n">
-        <v>0.09411727140347163</v>
+        <v>11854539.3985157</v>
       </c>
       <c r="E13" t="n">
-        <v>2.202183882395426</v>
+        <v>82.46804936726888</v>
+      </c>
+      <c r="F13" t="n">
+        <v>82.50361462817891</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>pines</t>
+          <t>doublewell2</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
+          <t>Kullback-Leibler</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
           <t>dds</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>424.0943400065104</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>5.336622873942058</v>
+      </c>
+      <c r="E14" t="n">
+        <v>7.27200984954834</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7.391373187863038</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>mcd</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>403.4309285481771</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>6.143062591552734</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7.268509705861409</v>
+      </c>
+      <c r="F15" t="n">
+        <v>7.389068510111819</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>pis</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>1051.229329427083</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>2.794068654378255</v>
+      </c>
+      <c r="E16" t="n">
+        <v>7.462174256642659</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7.590708826731253</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Log-variance</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5.432133992513021</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7.269322236378987</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7.393201273171556</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="n"/>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6.197343190511067</v>
+      </c>
+      <c r="E18" t="n">
+        <v>7.269106070200603</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.389769637086687</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2847549988.489681</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1540.305867513021</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1540.742386875876</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>funnel</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Kullback-Leibler</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.2376863161722819</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.142382979393005</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6.84800415950611</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.115148385365804</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.5960869590441386</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5.94196146465563</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1.403095761934916</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.446673075358073</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7.053018592034358</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Log-variance</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0.2837925752003987</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1.067343711853027</v>
+      </c>
+      <c r="F23" t="n">
+        <v>6.715308632988415</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="1" t="n"/>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.1046896775563558</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.6440276702245077</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5.944278317002742</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="1" t="n"/>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="n">
+        <v>13.3382862815232</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>gmmfixed</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Kullback-Leibler</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.4861413935820262</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.1514183580875397</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.147578732736723</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.5472275714079539</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.5548019607861837</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2.03095464980808</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n"/>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>3.305032968521118</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1.117149631182353</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2.071153409718854</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n"/>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>Log-variance</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1.974596063296</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1.87078579266866</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2.817087621699275</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n"/>
+      <c r="B30" s="1" t="n"/>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0.3242381314436595</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.1274864251414935</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.22698858951798</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="1" t="n"/>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5.820073286692302</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2.471234877904256</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2.865639303375772</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>pines</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Kullback-Leibler</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>402.2901713053386</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>405.8168334960938</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1086.773763020833</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>Log-variance</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>dds</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>874.6344604492188</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>mcd</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>272.8266906738281</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>pis</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2320.52978515625</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A14:A16"/>
+  <mergeCells count="18">
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A26:A31"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="A20:A25"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="A32:A37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>